<commit_message>
arayüz ve admin paneli güncellemeleri
</commit_message>
<xml_diff>
--- a/data/123.xlsx
+++ b/data/123.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\thomas\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586D45B2-0DB7-4CC3-8764-AFC7333907E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68D725D-1D98-4358-A10C-7BBDF42437E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1185" uniqueCount="781">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="780">
   <si>
     <t>NO</t>
   </si>
@@ -1383,9 +1383,6 @@
   </si>
   <si>
     <t>Peşimde olan saray görevlileri bisikletle Tahran'a geldiğim haberini alır almaz şaha ulaştırmış. Gelişimin yedinci gününde saraydan bir görevli şahın adına bana geliyor ve ertesi sabah 8'de beni "şahların şahı ve kralların kralı” ile görüşeceğim saraya götürmek üzere gönderilecek askerleri takip ederek kendisiyle birlikte Doshan tepedeki yaz sarayına kadar gitmemi rica ediyor. "Evet, elbette orada olmaktan ve Majestelerine Avrupa'dan gelen en son mucizeyi, muhteşem demir atı tanıtma vazifesini üstlenmekten son derece mutlu olacağım," yanıtını veriyorum ve görevli Fransız kibarlığıyla beni selamladıktan sonra ayrılıyor… Şahın gelmesini bekleyeceğimiz Doshan Tepe kapısına doğru ilerliyorum. Doshan Tepeden sonra yaklaşık 4 millik oldukça güzel bir yol kraliyet ailesine ait saraylara ve bahçelere çıkıyor. Majesteleri bu sabah Doshan Tepe'nin ilerisindeki dağlara atış yapmak için gidiyor ve benim de grupla birlikte birkaç mil sürmemi, böylece bisikletle yolculuk yapmanın nasıl bir şey olduğunu görmesi için güzel bir fırsat vermemi istiyor. Yavaş hareket eden şah beni ve büyük bir hizmetli grubunu kapıda tam bir saat bekletiyor. Kalabalığı arasında şahın baş avcısı da bulunuyor. Avcı beni bisiklete binerken görünce dengede durmanın nasıl mümkün olduğunu anlayamadığından, "ah muhteşem İngiliz," diye bağırıyor. Yaşlı avcının şaşkınlık sözlerini duyan herkes gülümsüyor ve şaka yoluyla gelecekte avlanma işini bisiklete binerek yapması gerektiğini tavsiye edip tekrar bisiklete binerek seleden ateş etmenin mümkün olduğunu direksiyonu tutmadan ilerleyerek gösterince atlılardan oluşan sevinçli kalabalık yürekten kahkahalar atıyor ve bazıları da "bravo, bravo" diye bağırıyor. Şahın arabası geldiği için herkes attan inip başını yere kadar eğiyor. Araba durup da şah beni ve tercümanı yanına çağırana kadar da öyle kalıyorlar. İki İngiliz arkadaşım bana şahtan ayrıldıktan sonra katılmayı planlayarak geri döndüğü için gruptaki tek Avrupalı benim.</t>
-  </si>
-  <si>
-    <t>167A169:G169</t>
   </si>
   <si>
     <t>Evet</t>
@@ -2509,7 +2506,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2557,19 +2554,16 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="12" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2823,11 +2817,11 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
+        <v>778</v>
+      </c>
+      <c r="G1" s="18" t="s">
         <v>779</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>780</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>5</v>
@@ -2865,11 +2859,11 @@
       <c r="E2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="19" t="s">
+        <v>461</v>
+      </c>
+      <c r="G2" s="19" t="s">
         <v>462</v>
-      </c>
-      <c r="G2" s="20" t="s">
-        <v>463</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>10</v>
@@ -2907,11 +2901,11 @@
       <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="21" t="s">
-        <v>443</v>
-      </c>
-      <c r="G3" s="22" t="s">
-        <v>464</v>
+      <c r="F3" s="20" t="s">
+        <v>442</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>463</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>10</v>
@@ -2949,11 +2943,11 @@
       <c r="E4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="21" t="s">
-        <v>444</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>465</v>
+      <c r="F4" s="20" t="s">
+        <v>443</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>464</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>10</v>
@@ -2991,11 +2985,11 @@
       <c r="E5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="21" t="s">
-        <v>445</v>
-      </c>
-      <c r="G5" s="21" t="s">
-        <v>466</v>
+      <c r="F5" s="20" t="s">
+        <v>444</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>465</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>10</v>
@@ -3033,11 +3027,11 @@
       <c r="E6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="21" t="s">
-        <v>446</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>467</v>
+      <c r="F6" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>466</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>10</v>
@@ -3075,11 +3069,11 @@
       <c r="E7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="21" t="s">
-        <v>447</v>
-      </c>
-      <c r="G7" s="21" t="s">
-        <v>468</v>
+      <c r="F7" s="20" t="s">
+        <v>446</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>467</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>10</v>
@@ -3117,11 +3111,11 @@
       <c r="E8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="21" t="s">
-        <v>448</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>469</v>
+      <c r="F8" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>468</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>10</v>
@@ -3159,11 +3153,11 @@
       <c r="E9" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="21" t="s">
-        <v>449</v>
-      </c>
-      <c r="G9" s="21" t="s">
-        <v>470</v>
+      <c r="F9" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>469</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>10</v>
@@ -3201,11 +3195,11 @@
       <c r="E10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F10" s="21" t="s">
-        <v>450</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>471</v>
+      <c r="F10" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>470</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>10</v>
@@ -3243,11 +3237,11 @@
       <c r="E11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="21" t="s">
-        <v>451</v>
-      </c>
-      <c r="G11" s="21" t="s">
-        <v>472</v>
+      <c r="F11" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>471</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>10</v>
@@ -3285,11 +3279,11 @@
       <c r="E12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="21" t="s">
-        <v>452</v>
-      </c>
-      <c r="G12" s="21" t="s">
-        <v>473</v>
+      <c r="F12" s="20" t="s">
+        <v>451</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>472</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>10</v>
@@ -3327,11 +3321,11 @@
       <c r="E13" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="21" t="s">
-        <v>453</v>
-      </c>
-      <c r="G13" s="21" t="s">
-        <v>474</v>
+      <c r="F13" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>473</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>10</v>
@@ -3369,11 +3363,11 @@
       <c r="E14" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="21" t="s">
-        <v>454</v>
-      </c>
-      <c r="G14" s="21" t="s">
-        <v>475</v>
+      <c r="F14" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>474</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>10</v>
@@ -3411,11 +3405,11 @@
       <c r="E15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="21" t="s">
-        <v>455</v>
-      </c>
-      <c r="G15" s="21" t="s">
-        <v>476</v>
+      <c r="F15" s="20" t="s">
+        <v>454</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>475</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>10</v>
@@ -3453,11 +3447,11 @@
       <c r="E16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F16" s="21" t="s">
-        <v>456</v>
-      </c>
-      <c r="G16" s="21" t="s">
-        <v>477</v>
+      <c r="F16" s="20" t="s">
+        <v>455</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>476</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>10</v>
@@ -3495,11 +3489,11 @@
       <c r="E17" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="21" t="s">
-        <v>457</v>
-      </c>
-      <c r="G17" s="21" t="s">
-        <v>478</v>
+      <c r="F17" s="20" t="s">
+        <v>456</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>477</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>10</v>
@@ -3537,11 +3531,11 @@
       <c r="E18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="21" t="s">
-        <v>458</v>
-      </c>
-      <c r="G18" s="21" t="s">
-        <v>479</v>
+      <c r="F18" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>478</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>10</v>
@@ -3579,11 +3573,11 @@
       <c r="E19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="21" t="s">
-        <v>459</v>
-      </c>
-      <c r="G19" s="21" t="s">
-        <v>480</v>
+      <c r="F19" s="20" t="s">
+        <v>458</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>479</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>10</v>
@@ -3621,11 +3615,11 @@
       <c r="E20" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="21" t="s">
-        <v>460</v>
-      </c>
-      <c r="G20" s="21" t="s">
-        <v>481</v>
+      <c r="F20" s="20" t="s">
+        <v>459</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>480</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>10</v>
@@ -3663,11 +3657,11 @@
       <c r="E21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F21" s="21" t="s">
-        <v>461</v>
-      </c>
-      <c r="G21" s="21" t="s">
-        <v>482</v>
+      <c r="F21" s="20" t="s">
+        <v>460</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>481</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>10</v>
@@ -3705,11 +3699,11 @@
       <c r="E22" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="21" t="s">
+      <c r="F22" s="20" t="s">
+        <v>482</v>
+      </c>
+      <c r="G22" s="20" t="s">
         <v>483</v>
-      </c>
-      <c r="G22" s="21" t="s">
-        <v>484</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>10</v>
@@ -3747,11 +3741,11 @@
       <c r="E23" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F23" s="21" t="s">
+      <c r="F23" s="20" t="s">
+        <v>484</v>
+      </c>
+      <c r="G23" s="20" t="s">
         <v>485</v>
-      </c>
-      <c r="G23" s="21" t="s">
-        <v>486</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>10</v>
@@ -3789,11 +3783,11 @@
       <c r="E24" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F24" s="21" t="s">
+      <c r="F24" s="20" t="s">
+        <v>486</v>
+      </c>
+      <c r="G24" s="20" t="s">
         <v>487</v>
-      </c>
-      <c r="G24" s="21" t="s">
-        <v>488</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>10</v>
@@ -3831,11 +3825,11 @@
       <c r="E25" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="20" t="s">
+        <v>488</v>
+      </c>
+      <c r="G25" s="20" t="s">
         <v>489</v>
-      </c>
-      <c r="G25" s="21" t="s">
-        <v>490</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>10</v>
@@ -3873,11 +3867,11 @@
       <c r="E26" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="20" t="s">
+        <v>490</v>
+      </c>
+      <c r="G26" s="20" t="s">
         <v>491</v>
-      </c>
-      <c r="G26" s="21" t="s">
-        <v>492</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>10</v>
@@ -3915,11 +3909,11 @@
       <c r="E27" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F27" s="21" t="s">
+      <c r="F27" s="20" t="s">
+        <v>492</v>
+      </c>
+      <c r="G27" s="20" t="s">
         <v>493</v>
-      </c>
-      <c r="G27" s="21" t="s">
-        <v>494</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>10</v>
@@ -3957,11 +3951,11 @@
       <c r="E28" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="20" t="s">
+        <v>494</v>
+      </c>
+      <c r="G28" s="20" t="s">
         <v>495</v>
-      </c>
-      <c r="G28" s="21" t="s">
-        <v>496</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>10</v>
@@ -3999,11 +3993,11 @@
       <c r="E29" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="F29" s="21" t="s">
+      <c r="F29" s="20" t="s">
+        <v>496</v>
+      </c>
+      <c r="G29" s="20" t="s">
         <v>497</v>
-      </c>
-      <c r="G29" s="21" t="s">
-        <v>498</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>10</v>
@@ -4041,11 +4035,11 @@
       <c r="E30" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F30" s="21" t="s">
+      <c r="F30" s="20" t="s">
+        <v>498</v>
+      </c>
+      <c r="G30" s="20" t="s">
         <v>499</v>
-      </c>
-      <c r="G30" s="21" t="s">
-        <v>500</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>10</v>
@@ -4083,11 +4077,11 @@
       <c r="E31" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F31" s="21" t="s">
+      <c r="F31" s="20" t="s">
+        <v>500</v>
+      </c>
+      <c r="G31" s="20" t="s">
         <v>501</v>
-      </c>
-      <c r="G31" s="21" t="s">
-        <v>502</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>10</v>
@@ -4125,11 +4119,11 @@
       <c r="E32" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="20" t="s">
+        <v>502</v>
+      </c>
+      <c r="G32" s="20" t="s">
         <v>503</v>
-      </c>
-      <c r="G32" s="21" t="s">
-        <v>504</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>10</v>
@@ -4167,11 +4161,11 @@
       <c r="E33" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="20" t="s">
+        <v>504</v>
+      </c>
+      <c r="G33" s="20" t="s">
         <v>505</v>
-      </c>
-      <c r="G33" s="21" t="s">
-        <v>506</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>10</v>
@@ -4209,11 +4203,11 @@
       <c r="E34" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="20" t="s">
+        <v>506</v>
+      </c>
+      <c r="G34" s="20" t="s">
         <v>507</v>
-      </c>
-      <c r="G34" s="21" t="s">
-        <v>508</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>10</v>
@@ -4251,11 +4245,11 @@
       <c r="E35" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="F35" s="21" t="s">
+      <c r="F35" s="20" t="s">
+        <v>508</v>
+      </c>
+      <c r="G35" s="20" t="s">
         <v>509</v>
-      </c>
-      <c r="G35" s="21" t="s">
-        <v>510</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>10</v>
@@ -4293,11 +4287,11 @@
       <c r="E36" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F36" s="20" t="s">
+        <v>510</v>
+      </c>
+      <c r="G36" s="20" t="s">
         <v>511</v>
-      </c>
-      <c r="G36" s="21" t="s">
-        <v>512</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>10</v>
@@ -4335,11 +4329,11 @@
       <c r="E37" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F37" s="21" t="s">
+      <c r="F37" s="20" t="s">
+        <v>512</v>
+      </c>
+      <c r="G37" s="20" t="s">
         <v>513</v>
-      </c>
-      <c r="G37" s="21" t="s">
-        <v>514</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>10</v>
@@ -4377,11 +4371,11 @@
       <c r="E38" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F38" s="21" t="s">
+      <c r="F38" s="20" t="s">
+        <v>514</v>
+      </c>
+      <c r="G38" s="20" t="s">
         <v>515</v>
-      </c>
-      <c r="G38" s="21" t="s">
-        <v>516</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>10</v>
@@ -4419,11 +4413,11 @@
       <c r="E39" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F39" s="21" t="s">
+      <c r="F39" s="20" t="s">
+        <v>516</v>
+      </c>
+      <c r="G39" s="20" t="s">
         <v>517</v>
-      </c>
-      <c r="G39" s="21" t="s">
-        <v>518</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>10</v>
@@ -4461,11 +4455,11 @@
       <c r="E40" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="21" t="s">
+      <c r="F40" s="20" t="s">
+        <v>518</v>
+      </c>
+      <c r="G40" s="20" t="s">
         <v>519</v>
-      </c>
-      <c r="G40" s="21" t="s">
-        <v>520</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>10</v>
@@ -4503,11 +4497,11 @@
       <c r="E41" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F41" s="21" t="s">
+      <c r="F41" s="20" t="s">
+        <v>520</v>
+      </c>
+      <c r="G41" s="20" t="s">
         <v>521</v>
-      </c>
-      <c r="G41" s="21" t="s">
-        <v>522</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>10</v>
@@ -4545,11 +4539,11 @@
       <c r="E42" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F42" s="21" t="s">
+      <c r="F42" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="G42" s="20" t="s">
         <v>523</v>
-      </c>
-      <c r="G42" s="21" t="s">
-        <v>524</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>10</v>
@@ -4587,11 +4581,11 @@
       <c r="E43" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F43" s="21" t="s">
+      <c r="F43" s="20" t="s">
+        <v>524</v>
+      </c>
+      <c r="G43" s="20" t="s">
         <v>525</v>
-      </c>
-      <c r="G43" s="21" t="s">
-        <v>526</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>10</v>
@@ -4629,11 +4623,11 @@
       <c r="E44" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="F44" s="21" t="s">
+      <c r="F44" s="20" t="s">
+        <v>526</v>
+      </c>
+      <c r="G44" s="20" t="s">
         <v>527</v>
-      </c>
-      <c r="G44" s="21" t="s">
-        <v>528</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>10</v>
@@ -4671,11 +4665,11 @@
       <c r="E45" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="F45" s="21" t="s">
+      <c r="F45" s="20" t="s">
+        <v>528</v>
+      </c>
+      <c r="G45" s="20" t="s">
         <v>529</v>
-      </c>
-      <c r="G45" s="21" t="s">
-        <v>530</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>10</v>
@@ -4713,11 +4707,11 @@
       <c r="E46" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F46" s="21" t="s">
+      <c r="F46" s="20" t="s">
+        <v>530</v>
+      </c>
+      <c r="G46" s="20" t="s">
         <v>531</v>
-      </c>
-      <c r="G46" s="21" t="s">
-        <v>532</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>10</v>
@@ -4755,11 +4749,11 @@
       <c r="E47" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="F47" s="21" t="s">
+      <c r="F47" s="20" t="s">
+        <v>532</v>
+      </c>
+      <c r="G47" s="20" t="s">
         <v>533</v>
-      </c>
-      <c r="G47" s="21" t="s">
-        <v>534</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>10</v>
@@ -4797,11 +4791,11 @@
       <c r="E48" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F48" s="21" t="s">
+      <c r="F48" s="20" t="s">
+        <v>534</v>
+      </c>
+      <c r="G48" s="20" t="s">
         <v>535</v>
-      </c>
-      <c r="G48" s="21" t="s">
-        <v>536</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>10</v>
@@ -4839,11 +4833,11 @@
       <c r="E49" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="F49" s="21" t="s">
+      <c r="F49" s="20" t="s">
+        <v>536</v>
+      </c>
+      <c r="G49" s="20" t="s">
         <v>537</v>
-      </c>
-      <c r="G49" s="21" t="s">
-        <v>538</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>10</v>
@@ -4881,11 +4875,11 @@
       <c r="E50" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="F50" s="21" t="s">
+      <c r="F50" s="20" t="s">
+        <v>538</v>
+      </c>
+      <c r="G50" s="20" t="s">
         <v>539</v>
-      </c>
-      <c r="G50" s="21" t="s">
-        <v>540</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>10</v>
@@ -4923,11 +4917,11 @@
       <c r="E51" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F51" s="21" t="s">
+      <c r="F51" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="G51" s="20" t="s">
         <v>541</v>
-      </c>
-      <c r="G51" s="21" t="s">
-        <v>542</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>10</v>
@@ -4965,11 +4959,11 @@
       <c r="E52" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="F52" s="21" t="s">
+      <c r="F52" s="20" t="s">
+        <v>542</v>
+      </c>
+      <c r="G52" s="20" t="s">
         <v>543</v>
-      </c>
-      <c r="G52" s="21" t="s">
-        <v>544</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>10</v>
@@ -5007,11 +5001,11 @@
       <c r="E53" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="F53" s="21" t="s">
+      <c r="F53" s="20" t="s">
+        <v>544</v>
+      </c>
+      <c r="G53" s="20" t="s">
         <v>545</v>
-      </c>
-      <c r="G53" s="21" t="s">
-        <v>546</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>10</v>
@@ -5049,11 +5043,11 @@
       <c r="E54" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="F54" s="21" t="s">
+      <c r="F54" s="20" t="s">
+        <v>546</v>
+      </c>
+      <c r="G54" s="20" t="s">
         <v>547</v>
-      </c>
-      <c r="G54" s="21" t="s">
-        <v>548</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>10</v>
@@ -5091,11 +5085,11 @@
       <c r="E55" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="F55" s="21" t="s">
+      <c r="F55" s="20" t="s">
+        <v>548</v>
+      </c>
+      <c r="G55" s="20" t="s">
         <v>549</v>
-      </c>
-      <c r="G55" s="21" t="s">
-        <v>550</v>
       </c>
       <c r="H55" s="6" t="s">
         <v>10</v>
@@ -5133,11 +5127,11 @@
       <c r="E56" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F56" s="21" t="s">
+      <c r="F56" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="G56" s="20" t="s">
         <v>551</v>
-      </c>
-      <c r="G56" s="21" t="s">
-        <v>552</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>10</v>
@@ -5175,11 +5169,11 @@
       <c r="E57" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="F57" s="21" t="s">
+      <c r="F57" s="20" t="s">
+        <v>552</v>
+      </c>
+      <c r="G57" s="20" t="s">
         <v>553</v>
-      </c>
-      <c r="G57" s="21" t="s">
-        <v>554</v>
       </c>
       <c r="H57" s="6" t="s">
         <v>10</v>
@@ -5217,11 +5211,11 @@
       <c r="E58" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F58" s="21" t="s">
+      <c r="F58" s="20" t="s">
+        <v>554</v>
+      </c>
+      <c r="G58" s="20" t="s">
         <v>555</v>
-      </c>
-      <c r="G58" s="21" t="s">
-        <v>556</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>10</v>
@@ -5259,11 +5253,11 @@
       <c r="E59" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="F59" s="21" t="s">
+      <c r="F59" s="20" t="s">
+        <v>556</v>
+      </c>
+      <c r="G59" s="20" t="s">
         <v>557</v>
-      </c>
-      <c r="G59" s="21" t="s">
-        <v>558</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>10</v>
@@ -5301,11 +5295,11 @@
       <c r="E60" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F60" s="21" t="s">
+      <c r="F60" s="20" t="s">
+        <v>558</v>
+      </c>
+      <c r="G60" s="20" t="s">
         <v>559</v>
-      </c>
-      <c r="G60" s="21" t="s">
-        <v>560</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>10</v>
@@ -5343,11 +5337,11 @@
       <c r="E61" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="F61" s="21" t="s">
+      <c r="F61" s="20" t="s">
+        <v>560</v>
+      </c>
+      <c r="G61" s="20" t="s">
         <v>561</v>
-      </c>
-      <c r="G61" s="21" t="s">
-        <v>562</v>
       </c>
       <c r="H61" s="6" t="s">
         <v>10</v>
@@ -5385,11 +5379,11 @@
       <c r="E62" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F62" s="21" t="s">
+      <c r="F62" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="G62" s="20" t="s">
         <v>563</v>
-      </c>
-      <c r="G62" s="21" t="s">
-        <v>564</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>10</v>
@@ -5427,11 +5421,11 @@
       <c r="E63" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="F63" s="21" t="s">
+      <c r="F63" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="G63" s="20" t="s">
         <v>565</v>
-      </c>
-      <c r="G63" s="21" t="s">
-        <v>566</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>10</v>
@@ -5469,11 +5463,11 @@
       <c r="E64" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="F64" s="21" t="s">
+      <c r="F64" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G64" s="20" t="s">
         <v>567</v>
-      </c>
-      <c r="G64" s="21" t="s">
-        <v>568</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>10</v>
@@ -5511,11 +5505,11 @@
       <c r="E65" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F65" s="21" t="s">
+      <c r="F65" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="G65" s="20" t="s">
         <v>569</v>
-      </c>
-      <c r="G65" s="21" t="s">
-        <v>570</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>10</v>
@@ -5553,11 +5547,11 @@
       <c r="E66" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="F66" s="21" t="s">
+      <c r="F66" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="G66" s="20" t="s">
         <v>571</v>
-      </c>
-      <c r="G66" s="21" t="s">
-        <v>572</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>10</v>
@@ -5595,11 +5589,11 @@
       <c r="E67" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="F67" s="21" t="s">
+      <c r="F67" s="20" t="s">
+        <v>572</v>
+      </c>
+      <c r="G67" s="20" t="s">
         <v>573</v>
-      </c>
-      <c r="G67" s="21" t="s">
-        <v>574</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>10</v>
@@ -5637,11 +5631,11 @@
       <c r="E68" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="F68" s="21" t="s">
+      <c r="F68" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="G68" s="20" t="s">
         <v>575</v>
-      </c>
-      <c r="G68" s="21" t="s">
-        <v>576</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>10</v>
@@ -5679,11 +5673,11 @@
       <c r="E69" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F69" s="21" t="s">
+      <c r="F69" s="20" t="s">
+        <v>576</v>
+      </c>
+      <c r="G69" s="20" t="s">
         <v>577</v>
-      </c>
-      <c r="G69" s="21" t="s">
-        <v>578</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>10</v>
@@ -5721,11 +5715,11 @@
       <c r="E70" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="F70" s="21" t="s">
+      <c r="F70" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="G70" s="20" t="s">
         <v>579</v>
-      </c>
-      <c r="G70" s="21" t="s">
-        <v>580</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>10</v>
@@ -5763,11 +5757,11 @@
       <c r="E71" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="F71" s="21" t="s">
+      <c r="F71" s="20" t="s">
+        <v>580</v>
+      </c>
+      <c r="G71" s="20" t="s">
         <v>581</v>
-      </c>
-      <c r="G71" s="21" t="s">
-        <v>582</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>10</v>
@@ -5805,11 +5799,11 @@
       <c r="E72" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="F72" s="21" t="s">
+      <c r="F72" s="20" t="s">
+        <v>582</v>
+      </c>
+      <c r="G72" s="20" t="s">
         <v>583</v>
-      </c>
-      <c r="G72" s="21" t="s">
-        <v>584</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>10</v>
@@ -5847,11 +5841,11 @@
       <c r="E73" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="F73" s="21" t="s">
+      <c r="F73" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="G73" s="20" t="s">
         <v>585</v>
-      </c>
-      <c r="G73" s="21" t="s">
-        <v>586</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>10</v>
@@ -5889,11 +5883,11 @@
       <c r="E74" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="F74" s="21" t="s">
+      <c r="F74" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="G74" s="20" t="s">
         <v>587</v>
-      </c>
-      <c r="G74" s="21" t="s">
-        <v>588</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>10</v>
@@ -5931,11 +5925,11 @@
       <c r="E75" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="F75" s="21" t="s">
+      <c r="F75" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="G75" s="20" t="s">
         <v>589</v>
-      </c>
-      <c r="G75" s="21" t="s">
-        <v>590</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>10</v>
@@ -5973,11 +5967,11 @@
       <c r="E76" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="F76" s="21" t="s">
+      <c r="F76" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="G76" s="20" t="s">
         <v>591</v>
-      </c>
-      <c r="G76" s="21" t="s">
-        <v>592</v>
       </c>
       <c r="H76" s="6" t="s">
         <v>10</v>
@@ -6015,11 +6009,11 @@
       <c r="E77" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="F77" s="21" t="s">
+      <c r="F77" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G77" s="20" t="s">
         <v>593</v>
-      </c>
-      <c r="G77" s="21" t="s">
-        <v>594</v>
       </c>
       <c r="H77" s="6" t="s">
         <v>10</v>
@@ -6057,11 +6051,11 @@
       <c r="E78" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="F78" s="21" t="s">
+      <c r="F78" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="G78" s="20" t="s">
         <v>595</v>
-      </c>
-      <c r="G78" s="21" t="s">
-        <v>596</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>10</v>
@@ -6099,11 +6093,11 @@
       <c r="E79" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F79" s="21" t="s">
+      <c r="F79" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="G79" s="20" t="s">
         <v>597</v>
-      </c>
-      <c r="G79" s="21" t="s">
-        <v>598</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>10</v>
@@ -6141,11 +6135,11 @@
       <c r="E80" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="F80" s="21" t="s">
+      <c r="F80" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G80" s="20" t="s">
         <v>599</v>
-      </c>
-      <c r="G80" s="21" t="s">
-        <v>600</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>10</v>
@@ -6183,11 +6177,11 @@
       <c r="E81" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="F81" s="21" t="s">
+      <c r="F81" s="20" t="s">
+        <v>600</v>
+      </c>
+      <c r="G81" s="20" t="s">
         <v>601</v>
-      </c>
-      <c r="G81" s="21" t="s">
-        <v>602</v>
       </c>
       <c r="H81" s="6" t="s">
         <v>10</v>
@@ -6225,11 +6219,11 @@
       <c r="E82" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="F82" s="21" t="s">
+      <c r="F82" s="20" t="s">
+        <v>602</v>
+      </c>
+      <c r="G82" s="20" t="s">
         <v>603</v>
-      </c>
-      <c r="G82" s="21" t="s">
-        <v>604</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>10</v>
@@ -6267,11 +6261,11 @@
       <c r="E83" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="F83" s="21" t="s">
+      <c r="F83" s="20" t="s">
+        <v>604</v>
+      </c>
+      <c r="G83" s="20" t="s">
         <v>605</v>
-      </c>
-      <c r="G83" s="21" t="s">
-        <v>606</v>
       </c>
       <c r="H83" s="6" t="s">
         <v>10</v>
@@ -6309,11 +6303,11 @@
       <c r="E84" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="F84" s="21" t="s">
+      <c r="F84" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="G84" s="20" t="s">
         <v>607</v>
-      </c>
-      <c r="G84" s="21" t="s">
-        <v>608</v>
       </c>
       <c r="H84" s="6" t="s">
         <v>10</v>
@@ -6351,11 +6345,11 @@
       <c r="E85" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="F85" s="21" t="s">
+      <c r="F85" s="20" t="s">
+        <v>608</v>
+      </c>
+      <c r="G85" s="20" t="s">
         <v>609</v>
-      </c>
-      <c r="G85" s="21" t="s">
-        <v>610</v>
       </c>
       <c r="H85" s="6" t="s">
         <v>10</v>
@@ -6393,11 +6387,11 @@
       <c r="E86" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="F86" s="21" t="s">
+      <c r="F86" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="G86" s="20" t="s">
         <v>611</v>
-      </c>
-      <c r="G86" s="21" t="s">
-        <v>612</v>
       </c>
       <c r="H86" s="6" t="s">
         <v>10</v>
@@ -6435,11 +6429,11 @@
       <c r="E87" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="F87" s="21" t="s">
+      <c r="F87" s="20" t="s">
+        <v>612</v>
+      </c>
+      <c r="G87" s="20" t="s">
         <v>613</v>
-      </c>
-      <c r="G87" s="21" t="s">
-        <v>614</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>10</v>
@@ -6477,11 +6471,11 @@
       <c r="E88" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F88" s="21" t="s">
+      <c r="F88" s="20" t="s">
+        <v>614</v>
+      </c>
+      <c r="G88" s="20" t="s">
         <v>615</v>
-      </c>
-      <c r="G88" s="21" t="s">
-        <v>616</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>10</v>
@@ -6519,11 +6513,11 @@
       <c r="E89" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="F89" s="21" t="s">
+      <c r="F89" s="20" t="s">
+        <v>616</v>
+      </c>
+      <c r="G89" s="20" t="s">
         <v>617</v>
-      </c>
-      <c r="G89" s="21" t="s">
-        <v>618</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>10</v>
@@ -6561,11 +6555,11 @@
       <c r="E90" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="F90" s="21" t="s">
+      <c r="F90" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="G90" s="20" t="s">
         <v>619</v>
-      </c>
-      <c r="G90" s="21" t="s">
-        <v>620</v>
       </c>
       <c r="H90" s="6" t="s">
         <v>10</v>
@@ -6603,11 +6597,11 @@
       <c r="E91" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="F91" s="21" t="s">
+      <c r="F91" s="20" t="s">
+        <v>620</v>
+      </c>
+      <c r="G91" s="20" t="s">
         <v>621</v>
-      </c>
-      <c r="G91" s="21" t="s">
-        <v>622</v>
       </c>
       <c r="H91" s="6" t="s">
         <v>10</v>
@@ -6645,11 +6639,11 @@
       <c r="E92" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="F92" s="21" t="s">
+      <c r="F92" s="20" t="s">
+        <v>622</v>
+      </c>
+      <c r="G92" s="20" t="s">
         <v>623</v>
-      </c>
-      <c r="G92" s="21" t="s">
-        <v>624</v>
       </c>
       <c r="H92" s="6" t="s">
         <v>10</v>
@@ -6687,11 +6681,11 @@
       <c r="E93" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="F93" s="21" t="s">
+      <c r="F93" s="20" t="s">
+        <v>624</v>
+      </c>
+      <c r="G93" s="20" t="s">
         <v>625</v>
-      </c>
-      <c r="G93" s="21" t="s">
-        <v>626</v>
       </c>
       <c r="H93" s="6" t="s">
         <v>10</v>
@@ -6729,11 +6723,11 @@
       <c r="E94" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="F94" s="21" t="s">
+      <c r="F94" s="20" t="s">
+        <v>626</v>
+      </c>
+      <c r="G94" s="20" t="s">
         <v>627</v>
-      </c>
-      <c r="G94" s="21" t="s">
-        <v>628</v>
       </c>
       <c r="H94" s="6" t="s">
         <v>10</v>
@@ -6771,11 +6765,11 @@
       <c r="E95" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="F95" s="21" t="s">
+      <c r="F95" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="G95" s="20" t="s">
         <v>629</v>
-      </c>
-      <c r="G95" s="21" t="s">
-        <v>630</v>
       </c>
       <c r="H95" s="6" t="s">
         <v>10</v>
@@ -6813,11 +6807,11 @@
       <c r="E96" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="F96" s="21" t="s">
+      <c r="F96" s="20" t="s">
+        <v>630</v>
+      </c>
+      <c r="G96" s="20" t="s">
         <v>631</v>
-      </c>
-      <c r="G96" s="21" t="s">
-        <v>632</v>
       </c>
       <c r="H96" s="6" t="s">
         <v>10</v>
@@ -6855,11 +6849,11 @@
       <c r="E97" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="F97" s="21" t="s">
+      <c r="F97" s="20" t="s">
+        <v>632</v>
+      </c>
+      <c r="G97" s="20" t="s">
         <v>633</v>
-      </c>
-      <c r="G97" s="21" t="s">
-        <v>634</v>
       </c>
       <c r="H97" s="6" t="s">
         <v>10</v>
@@ -6897,11 +6891,11 @@
       <c r="E98" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="F98" s="21" t="s">
+      <c r="F98" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="G98" s="20" t="s">
         <v>635</v>
-      </c>
-      <c r="G98" s="21" t="s">
-        <v>636</v>
       </c>
       <c r="H98" s="6" t="s">
         <v>10</v>
@@ -6939,14 +6933,14 @@
       <c r="E99" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="F99" s="21" t="s">
+      <c r="F99" s="20" t="s">
+        <v>636</v>
+      </c>
+      <c r="G99" s="20" t="s">
         <v>637</v>
       </c>
-      <c r="G99" s="21" t="s">
-        <v>638</v>
-      </c>
       <c r="H99" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I99" s="4"/>
       <c r="J99" s="4"/>
@@ -6981,14 +6975,14 @@
       <c r="E100" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="F100" s="21" t="s">
+      <c r="F100" s="20" t="s">
+        <v>638</v>
+      </c>
+      <c r="G100" s="20" t="s">
         <v>639</v>
       </c>
-      <c r="G100" s="21" t="s">
-        <v>640</v>
-      </c>
       <c r="H100" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I100" s="4"/>
       <c r="J100" s="4"/>
@@ -7023,14 +7017,14 @@
       <c r="E101" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="F101" s="21" t="s">
+      <c r="F101" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="G101" s="20" t="s">
         <v>641</v>
       </c>
-      <c r="G101" s="21" t="s">
-        <v>642</v>
-      </c>
       <c r="H101" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I101" s="4"/>
       <c r="J101" s="4"/>
@@ -7065,14 +7059,14 @@
       <c r="E102" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="F102" s="21" t="s">
+      <c r="F102" s="20" t="s">
+        <v>642</v>
+      </c>
+      <c r="G102" s="20" t="s">
         <v>643</v>
       </c>
-      <c r="G102" s="21" t="s">
-        <v>644</v>
-      </c>
       <c r="H102" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I102" s="4"/>
       <c r="J102" s="4"/>
@@ -7107,14 +7101,14 @@
       <c r="E103" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="F103" s="21" t="s">
+      <c r="F103" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="G103" s="20" t="s">
         <v>645</v>
       </c>
-      <c r="G103" s="21" t="s">
-        <v>646</v>
-      </c>
       <c r="H103" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I103" s="4"/>
       <c r="J103" s="4"/>
@@ -7149,14 +7143,14 @@
       <c r="E104" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="F104" s="21" t="s">
+      <c r="F104" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="G104" s="20" t="s">
         <v>647</v>
       </c>
-      <c r="G104" s="21" t="s">
-        <v>648</v>
-      </c>
       <c r="H104" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I104" s="4"/>
       <c r="J104" s="4"/>
@@ -7191,14 +7185,14 @@
       <c r="E105" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="F105" s="21" t="s">
+      <c r="F105" s="20" t="s">
+        <v>648</v>
+      </c>
+      <c r="G105" s="20" t="s">
         <v>649</v>
       </c>
-      <c r="G105" s="21" t="s">
-        <v>650</v>
-      </c>
       <c r="H105" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I105" s="4"/>
       <c r="J105" s="4"/>
@@ -7233,14 +7227,14 @@
       <c r="E106" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="F106" s="21" t="s">
+      <c r="F106" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="G106" s="20" t="s">
         <v>651</v>
       </c>
-      <c r="G106" s="21" t="s">
-        <v>652</v>
-      </c>
       <c r="H106" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I106" s="4"/>
       <c r="J106" s="4"/>
@@ -7275,14 +7269,14 @@
       <c r="E107" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="F107" s="21" t="s">
+      <c r="F107" s="20" t="s">
+        <v>652</v>
+      </c>
+      <c r="G107" s="20" t="s">
         <v>653</v>
       </c>
-      <c r="G107" s="21" t="s">
-        <v>654</v>
-      </c>
       <c r="H107" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I107" s="4"/>
       <c r="J107" s="4"/>
@@ -7317,14 +7311,14 @@
       <c r="E108" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="F108" s="21" t="s">
+      <c r="F108" s="20" t="s">
+        <v>654</v>
+      </c>
+      <c r="G108" s="20" t="s">
         <v>655</v>
       </c>
-      <c r="G108" s="21" t="s">
-        <v>656</v>
-      </c>
       <c r="H108" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I108" s="4"/>
       <c r="J108" s="4"/>
@@ -7359,11 +7353,11 @@
       <c r="E109" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="F109" s="21" t="s">
+      <c r="F109" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="G109" s="20" t="s">
         <v>657</v>
-      </c>
-      <c r="G109" s="21" t="s">
-        <v>658</v>
       </c>
       <c r="H109" s="6" t="s">
         <v>10</v>
@@ -7401,14 +7395,14 @@
       <c r="E110" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="F110" s="21" t="s">
+      <c r="F110" s="20" t="s">
+        <v>658</v>
+      </c>
+      <c r="G110" s="20" t="s">
         <v>659</v>
       </c>
-      <c r="G110" s="21" t="s">
-        <v>660</v>
-      </c>
       <c r="H110" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I110" s="4"/>
       <c r="J110" s="4"/>
@@ -7443,11 +7437,11 @@
       <c r="E111" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="F111" s="21" t="s">
+      <c r="F111" s="20" t="s">
+        <v>660</v>
+      </c>
+      <c r="G111" s="20" t="s">
         <v>661</v>
-      </c>
-      <c r="G111" s="21" t="s">
-        <v>662</v>
       </c>
       <c r="H111" s="6" t="s">
         <v>10</v>
@@ -7485,14 +7479,14 @@
       <c r="E112" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="F112" s="21" t="s">
+      <c r="F112" s="20" t="s">
+        <v>662</v>
+      </c>
+      <c r="G112" s="20" t="s">
         <v>663</v>
       </c>
-      <c r="G112" s="21" t="s">
-        <v>664</v>
-      </c>
       <c r="H112" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I112" s="4"/>
       <c r="J112" s="4"/>
@@ -7527,14 +7521,14 @@
       <c r="E113" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="F113" s="21" t="s">
+      <c r="F113" s="20" t="s">
+        <v>664</v>
+      </c>
+      <c r="G113" s="20" t="s">
         <v>665</v>
       </c>
-      <c r="G113" s="21" t="s">
-        <v>666</v>
-      </c>
       <c r="H113" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I113" s="4"/>
       <c r="J113" s="4"/>
@@ -7569,14 +7563,14 @@
       <c r="E114" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="F114" s="21" t="s">
+      <c r="F114" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="G114" s="20" t="s">
         <v>667</v>
       </c>
-      <c r="G114" s="21" t="s">
-        <v>668</v>
-      </c>
       <c r="H114" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I114" s="4"/>
       <c r="J114" s="4"/>
@@ -7611,14 +7605,14 @@
       <c r="E115" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="F115" s="21" t="s">
+      <c r="F115" s="20" t="s">
+        <v>668</v>
+      </c>
+      <c r="G115" s="20" t="s">
         <v>669</v>
       </c>
-      <c r="G115" s="21" t="s">
-        <v>670</v>
-      </c>
       <c r="H115" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I115" s="4"/>
       <c r="J115" s="4"/>
@@ -7653,14 +7647,14 @@
       <c r="E116" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="F116" s="21" t="s">
+      <c r="F116" s="20" t="s">
+        <v>670</v>
+      </c>
+      <c r="G116" s="20" t="s">
         <v>671</v>
       </c>
-      <c r="G116" s="21" t="s">
-        <v>672</v>
-      </c>
       <c r="H116" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I116" s="4"/>
       <c r="J116" s="4"/>
@@ -7695,14 +7689,14 @@
       <c r="E117" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="F117" s="21" t="s">
+      <c r="F117" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="G117" s="20" t="s">
         <v>673</v>
       </c>
-      <c r="G117" s="21" t="s">
-        <v>674</v>
-      </c>
       <c r="H117" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I117" s="4"/>
       <c r="J117" s="4"/>
@@ -7737,14 +7731,14 @@
       <c r="E118" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="F118" s="21" t="s">
+      <c r="F118" s="20" t="s">
+        <v>674</v>
+      </c>
+      <c r="G118" s="20" t="s">
         <v>675</v>
       </c>
-      <c r="G118" s="21" t="s">
-        <v>676</v>
-      </c>
       <c r="H118" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I118" s="4"/>
       <c r="J118" s="4"/>
@@ -7779,14 +7773,14 @@
       <c r="E119" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="F119" s="21" t="s">
+      <c r="F119" s="20" t="s">
+        <v>676</v>
+      </c>
+      <c r="G119" s="20" t="s">
         <v>677</v>
       </c>
-      <c r="G119" s="21" t="s">
-        <v>678</v>
-      </c>
       <c r="H119" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I119" s="4"/>
       <c r="J119" s="4"/>
@@ -7821,14 +7815,14 @@
       <c r="E120" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="F120" s="21" t="s">
+      <c r="F120" s="20" t="s">
+        <v>678</v>
+      </c>
+      <c r="G120" s="20" t="s">
         <v>679</v>
       </c>
-      <c r="G120" s="21" t="s">
-        <v>680</v>
-      </c>
       <c r="H120" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I120" s="4"/>
       <c r="J120" s="4"/>
@@ -7863,14 +7857,14 @@
       <c r="E121" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="F121" s="21" t="s">
+      <c r="F121" s="20" t="s">
+        <v>680</v>
+      </c>
+      <c r="G121" s="20" t="s">
         <v>681</v>
       </c>
-      <c r="G121" s="21" t="s">
-        <v>682</v>
-      </c>
       <c r="H121" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I121" s="4"/>
       <c r="J121" s="4"/>
@@ -7905,14 +7899,14 @@
       <c r="E122" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="F122" s="21" t="s">
+      <c r="F122" s="20" t="s">
+        <v>682</v>
+      </c>
+      <c r="G122" s="20" t="s">
         <v>683</v>
       </c>
-      <c r="G122" s="21" t="s">
-        <v>684</v>
-      </c>
       <c r="H122" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I122" s="4"/>
       <c r="J122" s="4"/>
@@ -7947,14 +7941,14 @@
       <c r="E123" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="F123" s="21" t="s">
+      <c r="F123" s="20" t="s">
+        <v>684</v>
+      </c>
+      <c r="G123" s="20" t="s">
         <v>685</v>
       </c>
-      <c r="G123" s="21" t="s">
-        <v>686</v>
-      </c>
       <c r="H123" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I123" s="4"/>
       <c r="J123" s="4"/>
@@ -7989,14 +7983,14 @@
       <c r="E124" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="F124" s="21" t="s">
+      <c r="F124" s="20" t="s">
+        <v>686</v>
+      </c>
+      <c r="G124" s="20" t="s">
         <v>687</v>
       </c>
-      <c r="G124" s="21" t="s">
-        <v>688</v>
-      </c>
       <c r="H124" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I124" s="4"/>
       <c r="J124" s="4"/>
@@ -8031,14 +8025,14 @@
       <c r="E125" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="F125" s="21" t="s">
+      <c r="F125" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="G125" s="20" t="s">
         <v>689</v>
       </c>
-      <c r="G125" s="21" t="s">
-        <v>690</v>
-      </c>
       <c r="H125" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I125" s="4"/>
       <c r="J125" s="4"/>
@@ -8073,14 +8067,14 @@
       <c r="E126" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="F126" s="21" t="s">
+      <c r="F126" s="20" t="s">
+        <v>690</v>
+      </c>
+      <c r="G126" s="20" t="s">
         <v>691</v>
       </c>
-      <c r="G126" s="21" t="s">
-        <v>692</v>
-      </c>
       <c r="H126" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I126" s="4"/>
       <c r="J126" s="4"/>
@@ -8115,14 +8109,14 @@
       <c r="E127" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="F127" s="21" t="s">
+      <c r="F127" s="20" t="s">
+        <v>692</v>
+      </c>
+      <c r="G127" s="20" t="s">
         <v>693</v>
       </c>
-      <c r="G127" s="21" t="s">
-        <v>694</v>
-      </c>
       <c r="H127" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
@@ -8157,14 +8151,14 @@
       <c r="E128" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="F128" s="21" t="s">
+      <c r="F128" s="20" t="s">
+        <v>694</v>
+      </c>
+      <c r="G128" s="20" t="s">
         <v>695</v>
       </c>
-      <c r="G128" s="21" t="s">
-        <v>696</v>
-      </c>
       <c r="H128" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I128" s="4"/>
       <c r="J128" s="4"/>
@@ -8199,14 +8193,14 @@
       <c r="E129" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="F129" s="21" t="s">
+      <c r="F129" s="20" t="s">
+        <v>696</v>
+      </c>
+      <c r="G129" s="20" t="s">
         <v>697</v>
       </c>
-      <c r="G129" s="21" t="s">
-        <v>698</v>
-      </c>
       <c r="H129" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I129" s="4"/>
       <c r="J129" s="4"/>
@@ -8241,14 +8235,14 @@
       <c r="E130" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="F130" s="21" t="s">
+      <c r="F130" s="20" t="s">
+        <v>698</v>
+      </c>
+      <c r="G130" s="20" t="s">
         <v>699</v>
       </c>
-      <c r="G130" s="21" t="s">
-        <v>700</v>
-      </c>
       <c r="H130" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I130" s="4"/>
       <c r="J130" s="4"/>
@@ -8283,14 +8277,14 @@
       <c r="E131" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="F131" s="21" t="s">
+      <c r="F131" s="20" t="s">
+        <v>700</v>
+      </c>
+      <c r="G131" s="20" t="s">
         <v>701</v>
       </c>
-      <c r="G131" s="21" t="s">
-        <v>702</v>
-      </c>
       <c r="H131" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I131" s="4"/>
       <c r="J131" s="4"/>
@@ -8325,14 +8319,14 @@
       <c r="E132" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="F132" s="21" t="s">
+      <c r="F132" s="20" t="s">
+        <v>702</v>
+      </c>
+      <c r="G132" s="20" t="s">
         <v>703</v>
       </c>
-      <c r="G132" s="21" t="s">
-        <v>704</v>
-      </c>
       <c r="H132" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I132" s="4"/>
       <c r="J132" s="4"/>
@@ -8367,14 +8361,14 @@
       <c r="E133" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="F133" s="21" t="s">
+      <c r="F133" s="20" t="s">
+        <v>704</v>
+      </c>
+      <c r="G133" s="20" t="s">
         <v>705</v>
       </c>
-      <c r="G133" s="21" t="s">
-        <v>706</v>
-      </c>
       <c r="H133" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I133" s="4"/>
       <c r="J133" s="4"/>
@@ -8409,14 +8403,14 @@
       <c r="E134" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="F134" s="21" t="s">
+      <c r="F134" s="20" t="s">
+        <v>706</v>
+      </c>
+      <c r="G134" s="20" t="s">
         <v>707</v>
       </c>
-      <c r="G134" s="21" t="s">
-        <v>708</v>
-      </c>
       <c r="H134" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I134" s="4"/>
       <c r="J134" s="4"/>
@@ -8451,14 +8445,14 @@
       <c r="E135" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="F135" s="21" t="s">
+      <c r="F135" s="20" t="s">
+        <v>708</v>
+      </c>
+      <c r="G135" s="20" t="s">
         <v>709</v>
       </c>
-      <c r="G135" s="21" t="s">
-        <v>710</v>
-      </c>
       <c r="H135" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I135" s="4"/>
       <c r="J135" s="4"/>
@@ -8493,14 +8487,14 @@
       <c r="E136" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="F136" s="21" t="s">
+      <c r="F136" s="20" t="s">
+        <v>710</v>
+      </c>
+      <c r="G136" s="20" t="s">
         <v>711</v>
       </c>
-      <c r="G136" s="21" t="s">
-        <v>712</v>
-      </c>
       <c r="H136" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I136" s="4"/>
       <c r="J136" s="4"/>
@@ -8535,14 +8529,14 @@
       <c r="E137" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="F137" s="21" t="s">
+      <c r="F137" s="20" t="s">
+        <v>712</v>
+      </c>
+      <c r="G137" s="20" t="s">
         <v>713</v>
       </c>
-      <c r="G137" s="21" t="s">
-        <v>714</v>
-      </c>
       <c r="H137" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I137" s="4"/>
       <c r="J137" s="4"/>
@@ -8577,14 +8571,14 @@
       <c r="E138" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="F138" s="21" t="s">
+      <c r="F138" s="20" t="s">
+        <v>714</v>
+      </c>
+      <c r="G138" s="20" t="s">
         <v>715</v>
       </c>
-      <c r="G138" s="21" t="s">
-        <v>716</v>
-      </c>
       <c r="H138" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I138" s="4"/>
       <c r="J138" s="4"/>
@@ -8619,14 +8613,14 @@
       <c r="E139" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="F139" s="21" t="s">
+      <c r="F139" s="20" t="s">
+        <v>716</v>
+      </c>
+      <c r="G139" s="20" t="s">
         <v>717</v>
       </c>
-      <c r="G139" s="21" t="s">
-        <v>718</v>
-      </c>
       <c r="H139" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I139" s="4"/>
       <c r="J139" s="4"/>
@@ -8661,14 +8655,14 @@
       <c r="E140" s="13" t="s">
         <v>371</v>
       </c>
-      <c r="F140" s="21" t="s">
+      <c r="F140" s="20" t="s">
+        <v>718</v>
+      </c>
+      <c r="G140" s="20" t="s">
         <v>719</v>
       </c>
-      <c r="G140" s="21" t="s">
-        <v>720</v>
-      </c>
       <c r="H140" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I140" s="4"/>
       <c r="J140" s="4"/>
@@ -8703,14 +8697,14 @@
       <c r="E141" s="13" t="s">
         <v>373</v>
       </c>
-      <c r="F141" s="21" t="s">
+      <c r="F141" s="20" t="s">
+        <v>720</v>
+      </c>
+      <c r="G141" s="20" t="s">
         <v>721</v>
       </c>
-      <c r="G141" s="21" t="s">
-        <v>722</v>
-      </c>
       <c r="H141" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I141" s="4"/>
       <c r="J141" s="4"/>
@@ -8745,14 +8739,14 @@
       <c r="E142" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="F142" s="21" t="s">
+      <c r="F142" s="20" t="s">
+        <v>722</v>
+      </c>
+      <c r="G142" s="20" t="s">
         <v>723</v>
       </c>
-      <c r="G142" s="21" t="s">
-        <v>724</v>
-      </c>
       <c r="H142" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I142" s="4"/>
       <c r="J142" s="4"/>
@@ -8787,14 +8781,14 @@
       <c r="E143" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="F143" s="21" t="s">
+      <c r="F143" s="20" t="s">
+        <v>724</v>
+      </c>
+      <c r="G143" s="20" t="s">
         <v>725</v>
       </c>
-      <c r="G143" s="21" t="s">
-        <v>726</v>
-      </c>
       <c r="H143" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I143" s="4"/>
       <c r="J143" s="4"/>
@@ -8829,14 +8823,14 @@
       <c r="E144" s="13" t="s">
         <v>381</v>
       </c>
-      <c r="F144" s="21" t="s">
+      <c r="F144" s="20" t="s">
+        <v>726</v>
+      </c>
+      <c r="G144" s="20" t="s">
         <v>727</v>
       </c>
-      <c r="G144" s="21" t="s">
-        <v>728</v>
-      </c>
       <c r="H144" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I144" s="4"/>
       <c r="J144" s="4"/>
@@ -8871,14 +8865,14 @@
       <c r="E145" s="13" t="s">
         <v>384</v>
       </c>
-      <c r="F145" s="21" t="s">
+      <c r="F145" s="20" t="s">
+        <v>728</v>
+      </c>
+      <c r="G145" s="20" t="s">
         <v>729</v>
       </c>
-      <c r="G145" s="21" t="s">
-        <v>730</v>
-      </c>
       <c r="H145" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I145" s="4"/>
       <c r="J145" s="4"/>
@@ -8913,14 +8907,14 @@
       <c r="E146" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="F146" s="21" t="s">
+      <c r="F146" s="20" t="s">
+        <v>730</v>
+      </c>
+      <c r="G146" s="20" t="s">
         <v>731</v>
       </c>
-      <c r="G146" s="21" t="s">
-        <v>732</v>
-      </c>
       <c r="H146" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I146" s="4"/>
       <c r="J146" s="4"/>
@@ -8955,14 +8949,14 @@
       <c r="E147" s="13" t="s">
         <v>389</v>
       </c>
-      <c r="F147" s="21" t="s">
+      <c r="F147" s="20" t="s">
+        <v>732</v>
+      </c>
+      <c r="G147" s="20" t="s">
         <v>733</v>
       </c>
-      <c r="G147" s="21" t="s">
-        <v>734</v>
-      </c>
       <c r="H147" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I147" s="4"/>
       <c r="J147" s="4"/>
@@ -8997,14 +8991,14 @@
       <c r="E148" s="13" t="s">
         <v>391</v>
       </c>
-      <c r="F148" s="21" t="s">
+      <c r="F148" s="20" t="s">
+        <v>734</v>
+      </c>
+      <c r="G148" s="20" t="s">
         <v>735</v>
       </c>
-      <c r="G148" s="21" t="s">
-        <v>736</v>
-      </c>
       <c r="H148" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I148" s="4"/>
       <c r="J148" s="4"/>
@@ -9039,14 +9033,14 @@
       <c r="E149" s="13" t="s">
         <v>393</v>
       </c>
-      <c r="F149" s="21" t="s">
+      <c r="F149" s="20" t="s">
+        <v>736</v>
+      </c>
+      <c r="G149" s="20" t="s">
         <v>737</v>
       </c>
-      <c r="G149" s="21" t="s">
-        <v>738</v>
-      </c>
       <c r="H149" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I149" s="4"/>
       <c r="J149" s="4"/>
@@ -9081,14 +9075,14 @@
       <c r="E150" s="13" t="s">
         <v>396</v>
       </c>
-      <c r="F150" s="21" t="s">
+      <c r="F150" s="20" t="s">
+        <v>738</v>
+      </c>
+      <c r="G150" s="20" t="s">
         <v>739</v>
       </c>
-      <c r="G150" s="21" t="s">
-        <v>740</v>
-      </c>
       <c r="H150" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I150" s="4"/>
       <c r="J150" s="4"/>
@@ -9123,14 +9117,14 @@
       <c r="E151" s="13" t="s">
         <v>399</v>
       </c>
-      <c r="F151" s="21" t="s">
+      <c r="F151" s="20" t="s">
+        <v>740</v>
+      </c>
+      <c r="G151" s="20" t="s">
         <v>741</v>
       </c>
-      <c r="G151" s="21" t="s">
-        <v>742</v>
-      </c>
       <c r="H151" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I151" s="4"/>
       <c r="J151" s="4"/>
@@ -9165,14 +9159,14 @@
       <c r="E152" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="F152" s="21" t="s">
+      <c r="F152" s="20" t="s">
+        <v>742</v>
+      </c>
+      <c r="G152" s="20" t="s">
         <v>743</v>
       </c>
-      <c r="G152" s="21" t="s">
-        <v>744</v>
-      </c>
       <c r="H152" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I152" s="4"/>
       <c r="J152" s="4"/>
@@ -9207,14 +9201,14 @@
       <c r="E153" s="13" t="s">
         <v>405</v>
       </c>
-      <c r="F153" s="21" t="s">
+      <c r="F153" s="20" t="s">
+        <v>744</v>
+      </c>
+      <c r="G153" s="20" t="s">
         <v>745</v>
       </c>
-      <c r="G153" s="21" t="s">
-        <v>746</v>
-      </c>
       <c r="H153" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I153" s="4"/>
       <c r="J153" s="4"/>
@@ -9249,14 +9243,14 @@
       <c r="E154" s="13" t="s">
         <v>407</v>
       </c>
-      <c r="F154" s="21" t="s">
+      <c r="F154" s="20" t="s">
+        <v>746</v>
+      </c>
+      <c r="G154" s="20" t="s">
         <v>747</v>
       </c>
-      <c r="G154" s="21" t="s">
-        <v>748</v>
-      </c>
       <c r="H154" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I154" s="4"/>
       <c r="J154" s="4"/>
@@ -9291,14 +9285,14 @@
       <c r="E155" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="F155" s="21" t="s">
+      <c r="F155" s="20" t="s">
+        <v>748</v>
+      </c>
+      <c r="G155" s="20" t="s">
         <v>749</v>
       </c>
-      <c r="G155" s="21" t="s">
-        <v>750</v>
-      </c>
       <c r="H155" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I155" s="4"/>
       <c r="J155" s="4"/>
@@ -9333,14 +9327,14 @@
       <c r="E156" s="13" t="s">
         <v>412</v>
       </c>
-      <c r="F156" s="21" t="s">
+      <c r="F156" s="20" t="s">
+        <v>750</v>
+      </c>
+      <c r="G156" s="20" t="s">
         <v>751</v>
       </c>
-      <c r="G156" s="21" t="s">
-        <v>752</v>
-      </c>
       <c r="H156" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I156" s="4"/>
       <c r="J156" s="4"/>
@@ -9375,14 +9369,14 @@
       <c r="E157" s="13" t="s">
         <v>414</v>
       </c>
-      <c r="F157" s="21" t="s">
+      <c r="F157" s="20" t="s">
+        <v>752</v>
+      </c>
+      <c r="G157" s="20" t="s">
         <v>753</v>
       </c>
-      <c r="G157" s="21" t="s">
-        <v>754</v>
-      </c>
       <c r="H157" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I157" s="4"/>
       <c r="J157" s="4"/>
@@ -9417,14 +9411,14 @@
       <c r="E158" s="13" t="s">
         <v>416</v>
       </c>
-      <c r="F158" s="21" t="s">
+      <c r="F158" s="20" t="s">
+        <v>754</v>
+      </c>
+      <c r="G158" s="20" t="s">
         <v>755</v>
       </c>
-      <c r="G158" s="21" t="s">
-        <v>756</v>
-      </c>
       <c r="H158" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I158" s="4"/>
       <c r="J158" s="4"/>
@@ -9459,11 +9453,11 @@
       <c r="E159" s="13" t="s">
         <v>418</v>
       </c>
-      <c r="F159" s="21" t="s">
+      <c r="F159" s="20" t="s">
+        <v>756</v>
+      </c>
+      <c r="G159" s="20" t="s">
         <v>757</v>
-      </c>
-      <c r="G159" s="21" t="s">
-        <v>758</v>
       </c>
       <c r="H159" s="6" t="s">
         <v>10</v>
@@ -9501,11 +9495,11 @@
       <c r="E160" s="13" t="s">
         <v>420</v>
       </c>
-      <c r="F160" s="21" t="s">
+      <c r="F160" s="20" t="s">
+        <v>758</v>
+      </c>
+      <c r="G160" s="20" t="s">
         <v>759</v>
-      </c>
-      <c r="G160" s="21" t="s">
-        <v>760</v>
       </c>
       <c r="H160" s="13" t="s">
         <v>10</v>
@@ -9543,11 +9537,11 @@
       <c r="E161" s="13" t="s">
         <v>422</v>
       </c>
-      <c r="F161" s="21" t="s">
+      <c r="F161" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="G161" s="20" t="s">
         <v>761</v>
-      </c>
-      <c r="G161" s="21" t="s">
-        <v>762</v>
       </c>
       <c r="H161" s="13" t="s">
         <v>10</v>
@@ -9585,11 +9579,11 @@
       <c r="E162" s="13" t="s">
         <v>424</v>
       </c>
-      <c r="F162" s="21" t="s">
+      <c r="F162" s="20" t="s">
+        <v>762</v>
+      </c>
+      <c r="G162" s="20" t="s">
         <v>763</v>
-      </c>
-      <c r="G162" s="21" t="s">
-        <v>764</v>
       </c>
       <c r="H162" s="13" t="s">
         <v>10</v>
@@ -9627,11 +9621,11 @@
       <c r="E163" s="13" t="s">
         <v>426</v>
       </c>
-      <c r="F163" s="21" t="s">
+      <c r="F163" s="20" t="s">
+        <v>764</v>
+      </c>
+      <c r="G163" s="20" t="s">
         <v>765</v>
-      </c>
-      <c r="G163" s="21" t="s">
-        <v>766</v>
       </c>
       <c r="H163" s="13" t="s">
         <v>10</v>
@@ -9669,11 +9663,11 @@
       <c r="E164" s="13" t="s">
         <v>428</v>
       </c>
-      <c r="F164" s="21" t="s">
+      <c r="F164" s="20" t="s">
+        <v>766</v>
+      </c>
+      <c r="G164" s="20" t="s">
         <v>767</v>
-      </c>
-      <c r="G164" s="21" t="s">
-        <v>768</v>
       </c>
       <c r="H164" s="13" t="s">
         <v>10</v>
@@ -9711,11 +9705,11 @@
       <c r="E165" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="F165" s="21" t="s">
+      <c r="F165" s="20" t="s">
+        <v>768</v>
+      </c>
+      <c r="G165" s="20" t="s">
         <v>769</v>
-      </c>
-      <c r="G165" s="21" t="s">
-        <v>770</v>
       </c>
       <c r="H165" s="13" t="s">
         <v>10</v>
@@ -9753,11 +9747,11 @@
       <c r="E166" s="13" t="s">
         <v>432</v>
       </c>
-      <c r="F166" s="21" t="s">
+      <c r="F166" s="20" t="s">
+        <v>770</v>
+      </c>
+      <c r="G166" s="20" t="s">
         <v>771</v>
-      </c>
-      <c r="G166" s="21" t="s">
-        <v>772</v>
       </c>
       <c r="H166" s="13" t="s">
         <v>10</v>
@@ -9795,11 +9789,11 @@
       <c r="E167" s="13" t="s">
         <v>435</v>
       </c>
-      <c r="F167" s="21" t="s">
+      <c r="F167" s="20" t="s">
+        <v>772</v>
+      </c>
+      <c r="G167" s="20" t="s">
         <v>773</v>
-      </c>
-      <c r="G167" s="21" t="s">
-        <v>774</v>
       </c>
       <c r="H167" s="13" t="s">
         <v>10</v>
@@ -9823,7 +9817,7 @@
     </row>
     <row r="168" spans="1:24" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B168" s="6" t="s">
         <v>436</v>
@@ -9837,11 +9831,11 @@
       <c r="E168" s="13" t="s">
         <v>437</v>
       </c>
-      <c r="F168" s="21" t="s">
+      <c r="F168" s="20" t="s">
+        <v>774</v>
+      </c>
+      <c r="G168" s="20" t="s">
         <v>775</v>
-      </c>
-      <c r="G168" s="21" t="s">
-        <v>776</v>
       </c>
       <c r="H168" s="13" t="s">
         <v>10</v>
@@ -9864,8 +9858,8 @@
       <c r="X168" s="4"/>
     </row>
     <row r="169" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A169" s="5" t="s">
-        <v>441</v>
+      <c r="A169" s="5">
+        <v>168</v>
       </c>
       <c r="B169" s="6" t="s">
         <v>438</v>
@@ -9879,11 +9873,11 @@
       <c r="E169" s="13" t="s">
         <v>440</v>
       </c>
-      <c r="F169" s="21" t="s">
+      <c r="F169" s="20" t="s">
+        <v>776</v>
+      </c>
+      <c r="G169" s="20" t="s">
         <v>777</v>
-      </c>
-      <c r="G169" s="21" t="s">
-        <v>778</v>
       </c>
       <c r="H169" s="13" t="s">
         <v>10</v>
@@ -9912,7 +9906,7 @@
       <c r="D170" s="13"/>
       <c r="E170" s="13"/>
       <c r="F170" s="15"/>
-      <c r="G170" s="17"/>
+      <c r="G170" s="4"/>
       <c r="H170" s="13"/>
       <c r="I170" s="4"/>
       <c r="J170" s="4"/>
@@ -9938,7 +9932,7 @@
       <c r="D171" s="13"/>
       <c r="E171" s="13"/>
       <c r="F171" s="15"/>
-      <c r="G171" s="17"/>
+      <c r="G171" s="4"/>
       <c r="H171" s="13"/>
       <c r="I171" s="4"/>
       <c r="J171" s="4"/>

</xml_diff>